<commit_message>
New visualizations with trimmed data
</commit_message>
<xml_diff>
--- a/data/smp_allocation.xlsx
+++ b/data/smp_allocation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jille\Documents\Uni\Master-Mechatronik\Masterarbeit\SMP-SignalProcessing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E27C4EF-C59A-42EC-A6FD-C130A5B9C057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649B114D-E5A3-4EFA-B74C-3DDDAA310A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{A2486933-0B32-43FE-AE21-582E25714C8B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A2486933-0B32-43FE-AE21-582E25714C8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>name</t>
   </si>
@@ -123,14 +123,28 @@
   </si>
   <si>
     <t>S45M1093</t>
+  </si>
+  <si>
+    <t>Surface</t>
+  </si>
+  <si>
+    <t>Ground</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -158,8 +172,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -494,10 +520,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA16F90C-85C8-49A9-BBE6-B7DFD4D049E3}">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -507,8 +533,14 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -518,8 +550,14 @@
       <c r="C2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -529,8 +567,14 @@
       <c r="C3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -540,8 +584,14 @@
       <c r="C4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -551,8 +601,14 @@
       <c r="C5">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5" s="2">
+        <v>100</v>
+      </c>
+      <c r="E5" s="3">
+        <v>11967024</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -562,8 +618,14 @@
       <c r="C6">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6" s="2">
+        <v>60.34</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1170.52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -573,8 +635,14 @@
       <c r="C7">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7" s="2">
+        <v>70.739999999999995</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -584,8 +652,14 @@
       <c r="C8">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8" s="2">
+        <v>57</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1170.3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -595,8 +669,14 @@
       <c r="C9">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D9" s="2">
+        <v>51.53</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1185.0899999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -606,8 +686,14 @@
       <c r="C10">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10" s="2">
+        <v>44</v>
+      </c>
+      <c r="E10" s="2">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -617,8 +703,14 @@
       <c r="C11">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11" s="2">
+        <v>46.3</v>
+      </c>
+      <c r="E11" s="2">
+        <v>1180.45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -628,8 +720,14 @@
       <c r="C12">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D12" s="2">
+        <v>53.94</v>
+      </c>
+      <c r="E12" s="2">
+        <v>1168.68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -639,8 +737,14 @@
       <c r="C13">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13" s="2">
+        <v>59.65</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1177</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -650,8 +754,14 @@
       <c r="C14">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D14" s="2">
+        <v>50.5</v>
+      </c>
+      <c r="E14" s="2">
+        <v>1177.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -661,8 +771,14 @@
       <c r="C15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D15" s="2">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -672,8 +788,14 @@
       <c r="C16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D16" s="2">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -683,8 +805,14 @@
       <c r="C17">
         <v>20</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D17" s="2">
+        <v>163</v>
+      </c>
+      <c r="E17" s="2">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -694,8 +822,14 @@
       <c r="C18">
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D18" s="2">
+        <v>140.5</v>
+      </c>
+      <c r="E18" s="2">
+        <v>892.53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -705,8 +839,14 @@
       <c r="C19">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D19" s="2">
+        <v>115</v>
+      </c>
+      <c r="E19" s="2">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -716,8 +856,14 @@
       <c r="C20">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D20" s="2">
+        <v>87.9</v>
+      </c>
+      <c r="E20" s="2">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -727,8 +873,14 @@
       <c r="C21">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D21" s="2">
+        <v>91.9</v>
+      </c>
+      <c r="E21" s="2">
+        <v>984.42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -738,8 +890,14 @@
       <c r="C22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D22" s="2">
+        <v>101.32</v>
+      </c>
+      <c r="E22" s="2">
+        <v>984.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -749,8 +907,14 @@
       <c r="C23">
         <v>8</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D23" s="2">
+        <v>54.4</v>
+      </c>
+      <c r="E23" s="3">
+        <v>856099</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -760,8 +924,14 @@
       <c r="C24">
         <v>8</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D24" s="2">
+        <v>80</v>
+      </c>
+      <c r="E24" s="2">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -771,8 +941,14 @@
       <c r="C25">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D25" s="2">
+        <v>45.5</v>
+      </c>
+      <c r="E25" s="2">
+        <v>931.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -782,8 +958,14 @@
       <c r="C26">
         <v>8</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D26" s="2">
+        <v>46.5</v>
+      </c>
+      <c r="E26" s="2">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -793,6 +975,104 @@
       <c r="C27">
         <v>8</v>
       </c>
+      <c r="D27" s="2">
+        <v>62.5</v>
+      </c>
+      <c r="E27" s="2">
+        <v>976.5</v>
+      </c>
+    </row>
+    <row r="34" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+    </row>
+    <row r="35" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+    </row>
+    <row r="36" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C38" s="2"/>
+      <c r="D38" s="3"/>
+    </row>
+    <row r="39" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+    </row>
+    <row r="45" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+    </row>
+    <row r="46" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+    </row>
+    <row r="47" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+    </row>
+    <row r="48" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+    </row>
+    <row r="49" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+    </row>
+    <row r="50" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+    </row>
+    <row r="51" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+    </row>
+    <row r="52" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C52" s="2"/>
+      <c r="D52" s="3"/>
+    </row>
+    <row r="53" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+    </row>
+    <row r="54" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+    </row>
+    <row r="55" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+    </row>
+    <row r="56" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixed trim with allocation table
</commit_message>
<xml_diff>
--- a/data/smp_allocation.xlsx
+++ b/data/smp_allocation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jille\Documents\Uni\Master-Mechatronik\Masterarbeit\SMP-SignalProcessing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649B114D-E5A3-4EFA-B74C-3DDDAA310A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EFA7D88-C248-46EF-99F5-5988091EE4B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A2486933-0B32-43FE-AE21-582E25714C8B}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{A2486933-0B32-43FE-AE21-582E25714C8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -911,7 +911,7 @@
         <v>54.4</v>
       </c>
       <c r="E23" s="3">
-        <v>856099</v>
+        <v>856</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
added plots for temperature
</commit_message>
<xml_diff>
--- a/data/smp_allocation.xlsx
+++ b/data/smp_allocation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jille\Documents\Uni\Master-Mechatronik\Masterarbeit\SMP-SignalProcessing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EFA7D88-C248-46EF-99F5-5988091EE4B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0412460B-B335-4D0E-99DA-4B883EF5D38F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{A2486933-0B32-43FE-AE21-582E25714C8B}"/>
   </bookViews>
@@ -571,7 +571,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="2">
-        <v>300</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -772,7 +772,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="2">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="E15" s="2">
         <v>300</v>
@@ -789,7 +789,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="2">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="E16" s="2">
         <v>300</v>

</xml_diff>